<commit_message>
Add structural profile reconciliation package
</commit_message>
<xml_diff>
--- a/research/structural-profiles-pilot/worksheet/structural_profiles_reference_and_owner_review.xlsx
+++ b/research/structural-profiles-pilot/worksheet/structural_profiles_reference_and_owner_review.xlsx
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Fable later proposes the seed coding. A blind independent model codes without seeing that submission. Codex later validates and produces a dimension-specific exception report. Jinhua reviews exceptions only. Domain experts later review all fusion rows and other routed cases.</t>
+          <t>The completed seed coding was produced in Claude Code using Claude Opus 5. The independent coding was produced by Codex using GPT-5.6 at extra-high reasoning effort. Fable remains the framework architect, not the row-level coder. Jinhua reviews routed exceptions only; domain experts later review all fusion rows and other routed cases.</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Send only fable_submission_template.xlsx to Fable. Send only blind_submission_template.xlsx to the blind model. Keep this owner workbook and all returned submissions out of the blind task.</t>
+          <t>The original Fable-named template is a historical handoff artifact. For reconciliation, use the immutable seed_submission_v1.csv and independent_submission_v1.csv copies pinned to their recorded PR heads.</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Absolute Fable-versus-independent difference is 2 or more on an S-dimension.</t>
+          <t>Absolute seed-versus-independent difference is 2 or more on an S-dimension.</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -6144,12 +6144,12 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="25" customWidth="1" min="15" max="15"/>
@@ -6199,32 +6199,32 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>fable_value</t>
+          <t>seed_value</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>blind_value</t>
+          <t>independent_value</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>fable_rationale</t>
+          <t>seed_rationale</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>blind_rationale</t>
+          <t>independent_rationale</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>fable_source_ids</t>
+          <t>seed_source_ids</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>blind_source_ids</t>
+          <t>independent_source_ids</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
@@ -8266,7 +8266,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="M4:M103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the canonical list or leave blank." promptTitle="Allowed values" prompt="Use a canonical allowed value. Blank remains allowed." type="list">
-      <formula1>"prefer_fable,prefer_independent,preserve_disagreement,needs_domain_review,needs_better_evidence"</formula1>
+      <formula1>"prefer_seed,prefer_independent,preserve_disagreement,needs_domain_review,needs_better_evidence"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the canonical list or leave blank." promptTitle="Allowed values" prompt="Use a canonical allowed value. Blank remains allowed." type="list">
       <formula1>"S1,S2,S3,S4,S5"</formula1>
@@ -15779,12 +15779,12 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>fable_value</t>
+          <t>seed_value</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>Fable value.</t>
+          <t>Seed value.</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr"/>
@@ -15807,12 +15807,12 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>blind_value</t>
+          <t>independent_value</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>Blind value.</t>
+          <t>Independent value.</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr"/>
@@ -15835,12 +15835,12 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>fable_rationale</t>
+          <t>seed_rationale</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>Fable rationale.</t>
+          <t>Seed rationale.</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr"/>
@@ -15863,12 +15863,12 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>blind_rationale</t>
+          <t>independent_rationale</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>Blind rationale.</t>
+          <t>Independent rationale.</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr"/>
@@ -15891,12 +15891,12 @@
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>fable_source_ids</t>
+          <t>seed_source_ids</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Fable source ids.</t>
+          <t>Seed source ids.</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr"/>
@@ -15919,12 +15919,12 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>blind_source_ids</t>
+          <t>independent_source_ids</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
         <is>
-          <t>Blind source ids.</t>
+          <t>Independent source ids.</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr"/>
@@ -15957,7 +15957,7 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>prefer_fable | prefer_independent | preserve_disagreement | needs_domain_review | needs_better_evidence</t>
+          <t>prefer_seed | prefer_independent | preserve_disagreement | needs_domain_review | needs_better_evidence</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr">

</xml_diff>